<commit_message>
data: publish 2026-09-25 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-25-182路.xlsx
+++ b/data/export/2026-09-25-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,33 +693,37 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>1/11</t>
         </is>
       </c>
     </row>
@@ -743,32 +751,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -776,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,33 +812,37 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>2/11</t>
         </is>
       </c>
     </row>
@@ -854,32 +870,36 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:39</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>79分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -887,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -911,33 +931,37 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>79.0</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>4/11</t>
         </is>
       </c>
     </row>
@@ -998,7 +1022,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1037,7 +1061,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
@@ -1048,7 +1072,7 @@
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1076,32 +1100,36 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>76分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -1109,7 +1137,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1133,33 +1161,37 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA6" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>76.0</t>
+        </is>
+      </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>3/11</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1252,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1302,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1363,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1413,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1421,22 @@
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>沪A13735A</t>
+          <t>沪A67026D</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>07:05</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1442,7 +1474,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1456,7 +1488,7 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:05</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -1492,7 +1524,911 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>1/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>2/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>79.0</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>4/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>76.0</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>3/11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-09-25 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-25-182路.xlsx
+++ b/data/export/2026-09-25-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC48"/>
+  <dimension ref="A1:AC52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>69.7</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>3/11</t>
+          <t>2/11</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -832,17 +832,17 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>72.2</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>3/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>2/11</t>
+          <t>3/11</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1194,12 +1194,12 @@
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>9/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>4/11</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1541,22 +1541,22 @@
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>10/11</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1665,17 +1665,17 @@
       </c>
       <c r="AA10" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>10/11</t>
+          <t>9/11</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>13:12</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1898,22 +1898,22 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA12" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>69.7</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>3/11</t>
+          <t>2/11</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2022,17 +2022,17 @@
       </c>
       <c r="AA13" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>72.2</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>3/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>69.8</t>
+          <t>69.2</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>2/11</t>
+          <t>3/11</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>9/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>4/11</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2846,22 +2846,22 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AA20" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="AC20" s="2" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>10/11</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>13:12</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA21" s="2" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3089,17 +3089,17 @@
       </c>
       <c r="AA22" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>10/11</t>
+          <t>9/11</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3208,17 +3208,17 @@
       </c>
       <c r="AA23" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>72.2</t>
         </is>
       </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>3/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
-          <t>69.8</t>
+          <t>69.2</t>
         </is>
       </c>
       <c r="AC24" s="2" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="Z25" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA25" s="2" t="inlineStr">
@@ -3521,7 +3521,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3570,12 +3570,12 @@
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC26" s="2" t="inlineStr">
         <is>
-          <t>9/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3694,7 @@
       </c>
       <c r="AC27" s="2" t="inlineStr">
         <is>
-          <t>2/11</t>
+          <t>3/11</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
       </c>
       <c r="AC28" s="2" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>4/11</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -4041,17 +4041,17 @@
       </c>
       <c r="AA30" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="AC30" s="2" t="inlineStr">
         <is>
-          <t>10/11</t>
+          <t>9/11</t>
         </is>
       </c>
     </row>
@@ -4116,7 +4116,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>13:12</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA31" s="2" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="Z32" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA32" s="2" t="inlineStr">
@@ -4354,7 +4354,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
-          <t>69.8</t>
+          <t>69.2</t>
         </is>
       </c>
       <c r="AC33" s="2" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="AC34" s="2" t="inlineStr">
         <is>
-          <t>2/11</t>
+          <t>3/11</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -4631,22 +4631,22 @@
       </c>
       <c r="Z35" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA35" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AA35" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="AC35" s="2" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>10/11</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4874,17 +4874,17 @@
       </c>
       <c r="AA37" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>72.2</t>
         </is>
       </c>
       <c r="AC37" s="2" t="inlineStr">
         <is>
-          <t>3/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -4949,7 +4949,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>13:12</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4988,7 +4988,7 @@
       </c>
       <c r="Z38" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA38" s="2" t="inlineStr">
@@ -5041,24 +5041,24 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>71分钟</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5117,12 +5117,12 @@
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC39" s="2" t="inlineStr">
         <is>
-          <t>9/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -5160,24 +5160,24 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>72分钟</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
-          <t>69.8</t>
+          <t>69.2</t>
         </is>
       </c>
       <c r="AC40" s="2" t="inlineStr">
@@ -5269,32 +5269,36 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -5302,7 +5306,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -5326,17 +5330,17 @@
       </c>
       <c r="W41" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X41" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z41" s="2" t="inlineStr">
@@ -5346,17 +5350,17 @@
       </c>
       <c r="AA41" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="AC41" s="2" t="inlineStr">
         <is>
-          <t>10/11</t>
+          <t>9/11</t>
         </is>
       </c>
     </row>
@@ -5384,32 +5388,36 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>14:22</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>79分钟</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -5417,7 +5425,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5441,37 +5449,37 @@
       </c>
       <c r="W42" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z42" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AA42" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="AC42" s="2" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>10/11</t>
         </is>
       </c>
     </row>
@@ -5499,32 +5507,36 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M43" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -5532,7 +5544,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -5556,37 +5568,37 @@
       </c>
       <c r="W43" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X43" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y43" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z43" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA43" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA43" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>69.7</t>
         </is>
       </c>
       <c r="AC43" s="2" t="inlineStr">
         <is>
-          <t>3/11</t>
+          <t>2/11</t>
         </is>
       </c>
     </row>
@@ -5614,32 +5626,36 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>79分钟</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -5647,7 +5663,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5671,17 +5687,17 @@
       </c>
       <c r="W44" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X44" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y44" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z44" s="2" t="inlineStr">
@@ -5691,17 +5707,17 @@
       </c>
       <c r="AA44" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>72.2</t>
         </is>
       </c>
       <c r="AC44" s="2" t="inlineStr">
         <is>
-          <t>3/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -5762,7 +5778,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -5801,7 +5817,7 @@
       </c>
       <c r="Z45" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA45" s="2" t="inlineStr">
@@ -5877,7 +5893,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -5926,12 +5942,12 @@
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC46" s="2" t="inlineStr">
         <is>
-          <t>9/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -5992,7 +6008,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -6107,7 +6123,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6151,17 +6167,477 @@
       </c>
       <c r="AA48" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB48" s="2" t="inlineStr">
+        <is>
+          <t>73.2</t>
+        </is>
+      </c>
+      <c r="AC48" s="2" t="inlineStr">
+        <is>
+          <t>9/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>14:52</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="inlineStr"/>
+      <c r="R49" s="2" t="inlineStr"/>
+      <c r="S49" s="2" t="inlineStr"/>
+      <c r="T49" s="2" t="inlineStr"/>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>14:52</t>
+        </is>
+      </c>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W49" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X49" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y49" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB49" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
+      <c r="AC49" s="2" t="inlineStr">
+        <is>
+          <t>10/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr"/>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="inlineStr"/>
+      <c r="R50" s="2" t="inlineStr"/>
+      <c r="S50" s="2" t="inlineStr"/>
+      <c r="T50" s="2" t="inlineStr"/>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W50" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y50" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z50" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA50" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AB48" s="2" t="inlineStr">
-        <is>
-          <t>73.3</t>
-        </is>
-      </c>
-      <c r="AC48" s="2" t="inlineStr">
-        <is>
-          <t>10/11</t>
+      <c r="AB50" s="2" t="inlineStr">
+        <is>
+          <t>69.7</t>
+        </is>
+      </c>
+      <c r="AC50" s="2" t="inlineStr">
+        <is>
+          <t>2/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr"/>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q51" s="2" t="inlineStr"/>
+      <c r="R51" s="2" t="inlineStr"/>
+      <c r="S51" s="2" t="inlineStr"/>
+      <c r="T51" s="2" t="inlineStr"/>
+      <c r="U51" s="2" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W51" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y51" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z51" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA51" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB51" s="2" t="inlineStr">
+        <is>
+          <t>72.8</t>
+        </is>
+      </c>
+      <c r="AC51" s="2" t="inlineStr">
+        <is>
+          <t>7/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr"/>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="inlineStr"/>
+      <c r="R52" s="2" t="inlineStr"/>
+      <c r="S52" s="2" t="inlineStr"/>
+      <c r="T52" s="2" t="inlineStr"/>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W52" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X52" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y52" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z52" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AA52" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB52" s="2" t="inlineStr">
+        <is>
+          <t>72.8</t>
+        </is>
+      </c>
+      <c r="AC52" s="2" t="inlineStr">
+        <is>
+          <t>7/11</t>
         </is>
       </c>
     </row>

</xml_diff>